<commit_message>
teste pra ver qual o problema do Render
</commit_message>
<xml_diff>
--- a/temporario/16-07-2026_Noite.xlsx
+++ b/temporario/16-07-2026_Noite.xlsx
@@ -15,9 +15,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="10">
     <font>
@@ -382,7 +381,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="63">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -514,7 +513,7 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="8" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -533,6 +532,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -634,6 +636,9 @@
       </blipFill>
       <spPr>
         <a:prstGeom prst="rect"/>
+        <a:ln>
+          <a:prstDash val="solid"/>
+        </a:ln>
       </spPr>
     </pic>
     <clientData/>
@@ -843,7 +848,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AG30"/>
+  <dimension ref="A1:AG40"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col width="1.42578125" customWidth="1" min="1" max="1"/>
@@ -929,7 +934,7 @@
           <t>DATA:</t>
         </is>
       </c>
-      <c r="D3" s="51" t="n">
+      <c r="D3" s="62" t="n">
         <v>46219</v>
       </c>
       <c r="E3" s="9" t="inlineStr">
@@ -1154,13 +1159,14 @@
       <c r="S6" s="60" t="inlineStr"/>
       <c r="T6" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 07EBAC78</t>
+          <t>LUARI - 17391612</t>
         </is>
       </c>
       <c r="U6" s="60" t="inlineStr"/>
       <c r="V6" s="60" t="inlineStr"/>
       <c r="W6" s="60" t="inlineStr"/>
     </row>
+    <row r="7"/>
     <row r="8">
       <c r="C8" s="60" t="inlineStr">
         <is>
@@ -1172,11 +1178,31 @@
           <t>26/02258</t>
         </is>
       </c>
-      <c r="E8" s="60" t="inlineStr"/>
-      <c r="F8" s="60" t="inlineStr"/>
-      <c r="G8" s="60" t="inlineStr"/>
-      <c r="H8" s="60" t="inlineStr"/>
-      <c r="I8" s="60" t="inlineStr"/>
+      <c r="E8" s="60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="F8" s="60" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="G8" s="60" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+      <c r="H8" s="60" t="inlineStr">
+        <is>
+          <t>52852787</t>
+        </is>
+      </c>
+      <c r="I8" s="60" t="inlineStr">
+        <is>
+          <t>527878</t>
+        </is>
+      </c>
       <c r="J8" s="60" t="inlineStr">
         <is>
           <t>CASA MAIS</t>
@@ -1217,13 +1243,14 @@
       <c r="S8" s="60" t="inlineStr"/>
       <c r="T8" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 01175496</t>
+          <t>LUARI - 27D1B044</t>
         </is>
       </c>
       <c r="U8" s="60" t="inlineStr"/>
       <c r="V8" s="60" t="inlineStr"/>
       <c r="W8" s="60" t="inlineStr"/>
     </row>
+    <row r="9"/>
     <row r="10">
       <c r="C10" s="60" t="inlineStr">
         <is>
@@ -1281,13 +1308,14 @@
       <c r="S10" s="60" t="inlineStr"/>
       <c r="T10" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 9C0971D7</t>
+          <t>LUARI - 912A0264</t>
         </is>
       </c>
       <c r="U10" s="60" t="inlineStr"/>
       <c r="V10" s="60" t="inlineStr"/>
       <c r="W10" s="60" t="inlineStr"/>
     </row>
+    <row r="11"/>
     <row r="12">
       <c r="C12" s="60" t="inlineStr">
         <is>
@@ -1340,13 +1368,14 @@
       <c r="S12" s="60" t="inlineStr"/>
       <c r="T12" s="60" t="inlineStr">
         <is>
-          <t>LUARI - E5308147</t>
+          <t>LUARI - 3B8DE027</t>
         </is>
       </c>
       <c r="U12" s="60" t="inlineStr"/>
       <c r="V12" s="60" t="inlineStr"/>
       <c r="W12" s="60" t="inlineStr"/>
     </row>
+    <row r="13"/>
     <row r="14">
       <c r="C14" s="60" t="n">
         <v>24282</v>
@@ -1397,13 +1426,14 @@
       <c r="S14" s="60" t="inlineStr"/>
       <c r="T14" s="60" t="inlineStr">
         <is>
-          <t>LUARI - D8F7B46A</t>
+          <t>LUARI - 12C40B80</t>
         </is>
       </c>
       <c r="U14" s="60" t="inlineStr"/>
       <c r="V14" s="60" t="inlineStr"/>
       <c r="W14" s="60" t="inlineStr"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="C16" s="60" t="inlineStr">
         <is>
@@ -1452,13 +1482,14 @@
       <c r="S16" s="60" t="inlineStr"/>
       <c r="T16" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 06B5B0DD</t>
+          <t>LUARI - A9A5180E</t>
         </is>
       </c>
       <c r="U16" s="60" t="inlineStr"/>
       <c r="V16" s="60" t="inlineStr"/>
       <c r="W16" s="60" t="inlineStr"/>
     </row>
+    <row r="17"/>
     <row r="18">
       <c r="C18" s="60" t="inlineStr">
         <is>
@@ -1511,13 +1542,14 @@
       <c r="S18" s="60" t="inlineStr"/>
       <c r="T18" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 11008E44</t>
+          <t>LUARI - 2EB753A3</t>
         </is>
       </c>
       <c r="U18" s="60" t="inlineStr"/>
       <c r="V18" s="60" t="inlineStr"/>
       <c r="W18" s="60" t="inlineStr"/>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="C20" s="60" t="inlineStr">
         <is>
@@ -1570,13 +1602,14 @@
       <c r="S20" s="60" t="inlineStr"/>
       <c r="T20" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 53913B95</t>
+          <t>LUARI - 8C917472</t>
         </is>
       </c>
       <c r="U20" s="60" t="inlineStr"/>
       <c r="V20" s="60" t="inlineStr"/>
       <c r="W20" s="60" t="inlineStr"/>
     </row>
+    <row r="21"/>
     <row r="22">
       <c r="C22" s="60" t="inlineStr">
         <is>
@@ -1629,13 +1662,14 @@
       <c r="S22" s="60" t="inlineStr"/>
       <c r="T22" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 5946A8C1</t>
+          <t>LUARI - 166C5ED4</t>
         </is>
       </c>
       <c r="U22" s="60" t="inlineStr"/>
       <c r="V22" s="60" t="inlineStr"/>
       <c r="W22" s="60" t="inlineStr"/>
     </row>
+    <row r="23"/>
     <row r="24">
       <c r="C24" s="60" t="inlineStr">
         <is>
@@ -1684,13 +1718,14 @@
       <c r="S24" s="60" t="inlineStr"/>
       <c r="T24" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 5ADC0D8F</t>
+          <t>LUARI - BD69F505</t>
         </is>
       </c>
       <c r="U24" s="60" t="inlineStr"/>
       <c r="V24" s="60" t="inlineStr"/>
       <c r="W24" s="60" t="inlineStr"/>
     </row>
+    <row r="25"/>
     <row r="26">
       <c r="C26" s="60" t="n">
         <v>22660</v>
@@ -1700,11 +1735,31 @@
           <t>26/02260</t>
         </is>
       </c>
-      <c r="E26" s="60" t="inlineStr"/>
-      <c r="F26" s="60" t="inlineStr"/>
-      <c r="G26" s="60" t="inlineStr"/>
-      <c r="H26" s="60" t="inlineStr"/>
-      <c r="I26" s="60" t="inlineStr"/>
+      <c r="E26" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F26" s="60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+      <c r="G26" s="60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="H26" s="60" t="inlineStr">
+        <is>
+          <t>016561</t>
+        </is>
+      </c>
+      <c r="I26" s="60" t="inlineStr">
+        <is>
+          <t>65666</t>
+        </is>
+      </c>
       <c r="J26" s="60" t="inlineStr">
         <is>
           <t>CATUPIRY - SANTA VITORIA</t>
@@ -1745,13 +1800,14 @@
       <c r="S26" s="60" t="inlineStr"/>
       <c r="T26" s="60" t="inlineStr">
         <is>
-          <t>LUARI - F139EA32</t>
+          <t>LUARI - 7181FFBF</t>
         </is>
       </c>
       <c r="U26" s="60" t="inlineStr"/>
       <c r="V26" s="60" t="inlineStr"/>
       <c r="W26" s="60" t="inlineStr"/>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="C28" s="60" t="inlineStr">
         <is>
@@ -1808,13 +1864,14 @@
       <c r="S28" s="60" t="inlineStr"/>
       <c r="T28" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 70AC39F8</t>
+          <t>LUARI - F7BE0030</t>
         </is>
       </c>
       <c r="U28" s="60" t="inlineStr"/>
       <c r="V28" s="60" t="inlineStr"/>
       <c r="W28" s="60" t="inlineStr"/>
     </row>
+    <row r="29"/>
     <row r="30">
       <c r="C30" s="60" t="inlineStr">
         <is>
@@ -1871,12 +1928,342 @@
       <c r="S30" s="60" t="inlineStr"/>
       <c r="T30" s="60" t="inlineStr">
         <is>
-          <t>LUARI - 4E2D026C</t>
+          <t>LUARI - FA1A1322</t>
         </is>
       </c>
       <c r="U30" s="60" t="inlineStr"/>
       <c r="V30" s="60" t="inlineStr"/>
       <c r="W30" s="60" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="Q31" s="60" t="inlineStr">
+        <is>
+          <t>26/02260</t>
+        </is>
+      </c>
+      <c r="R31" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S31" s="60" t="inlineStr">
+        <is>
+          <t>16:13:39</t>
+        </is>
+      </c>
+      <c r="T31" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 7181FFBF</t>
+        </is>
+      </c>
+      <c r="U31" s="60" t="inlineStr">
+        <is>
+          <t>pesagem</t>
+        </is>
+      </c>
+      <c r="V31" s="60" t="n"/>
+      <c r="W31" s="60" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="Q32" s="60" t="inlineStr">
+        <is>
+          <t>26/02260</t>
+        </is>
+      </c>
+      <c r="R32" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S32" s="60" t="inlineStr">
+        <is>
+          <t>16:13:39</t>
+        </is>
+      </c>
+      <c r="T32" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 7181FFBF</t>
+        </is>
+      </c>
+      <c r="U32" s="60" t="inlineStr">
+        <is>
+          <t>pesagem</t>
+        </is>
+      </c>
+      <c r="V32" s="60" t="n"/>
+      <c r="W32" s="60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="Q33" s="60" t="inlineStr">
+        <is>
+          <t>26/02260</t>
+        </is>
+      </c>
+      <c r="R33" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S33" s="60" t="inlineStr">
+        <is>
+          <t>16:13:39</t>
+        </is>
+      </c>
+      <c r="T33" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 7181FFBF</t>
+        </is>
+      </c>
+      <c r="U33" s="60" t="inlineStr">
+        <is>
+          <t>pesagem</t>
+        </is>
+      </c>
+      <c r="V33" s="60" t="n"/>
+      <c r="W33" s="60" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="Q34" s="60" t="inlineStr">
+        <is>
+          <t>26/02260</t>
+        </is>
+      </c>
+      <c r="R34" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S34" s="60" t="inlineStr">
+        <is>
+          <t>16:13:39</t>
+        </is>
+      </c>
+      <c r="T34" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 7181FFBF</t>
+        </is>
+      </c>
+      <c r="U34" s="60" t="inlineStr">
+        <is>
+          <t>pesagem</t>
+        </is>
+      </c>
+      <c r="V34" s="60" t="n"/>
+      <c r="W34" s="60" t="inlineStr">
+        <is>
+          <t>016561</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="Q35" s="60" t="inlineStr">
+        <is>
+          <t>26/02260</t>
+        </is>
+      </c>
+      <c r="R35" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S35" s="60" t="inlineStr">
+        <is>
+          <t>16:13:39</t>
+        </is>
+      </c>
+      <c r="T35" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 7181FFBF</t>
+        </is>
+      </c>
+      <c r="U35" s="60" t="inlineStr">
+        <is>
+          <t>pesagem</t>
+        </is>
+      </c>
+      <c r="V35" s="60" t="n"/>
+      <c r="W35" s="60" t="inlineStr">
+        <is>
+          <t>65666</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="Q36" s="60" t="inlineStr">
+        <is>
+          <t>26/02258</t>
+        </is>
+      </c>
+      <c r="R36" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S36" s="60" t="inlineStr">
+        <is>
+          <t>16:14:00</t>
+        </is>
+      </c>
+      <c r="T36" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 27D1B044</t>
+        </is>
+      </c>
+      <c r="U36" s="60" t="inlineStr">
+        <is>
+          <t>atualizacao</t>
+        </is>
+      </c>
+      <c r="V36" s="60" t="n"/>
+      <c r="W36" s="60" t="inlineStr">
+        <is>
+          <t>4</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="Q37" s="60" t="inlineStr">
+        <is>
+          <t>26/02258</t>
+        </is>
+      </c>
+      <c r="R37" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S37" s="60" t="inlineStr">
+        <is>
+          <t>16:14:00</t>
+        </is>
+      </c>
+      <c r="T37" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 27D1B044</t>
+        </is>
+      </c>
+      <c r="U37" s="60" t="inlineStr">
+        <is>
+          <t>atualizacao</t>
+        </is>
+      </c>
+      <c r="V37" s="60" t="n"/>
+      <c r="W37" s="60" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="Q38" s="60" t="inlineStr">
+        <is>
+          <t>26/02258</t>
+        </is>
+      </c>
+      <c r="R38" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S38" s="60" t="inlineStr">
+        <is>
+          <t>16:14:00</t>
+        </is>
+      </c>
+      <c r="T38" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 27D1B044</t>
+        </is>
+      </c>
+      <c r="U38" s="60" t="inlineStr">
+        <is>
+          <t>atualizacao</t>
+        </is>
+      </c>
+      <c r="V38" s="60" t="n"/>
+      <c r="W38" s="60" t="inlineStr">
+        <is>
+          <t>85</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="Q39" s="60" t="inlineStr">
+        <is>
+          <t>26/02258</t>
+        </is>
+      </c>
+      <c r="R39" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S39" s="60" t="inlineStr">
+        <is>
+          <t>16:14:00</t>
+        </is>
+      </c>
+      <c r="T39" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 27D1B044</t>
+        </is>
+      </c>
+      <c r="U39" s="60" t="inlineStr">
+        <is>
+          <t>atualizacao</t>
+        </is>
+      </c>
+      <c r="V39" s="60" t="n"/>
+      <c r="W39" s="60" t="inlineStr">
+        <is>
+          <t>52852787</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="Q40" s="60" t="inlineStr">
+        <is>
+          <t>26/02258</t>
+        </is>
+      </c>
+      <c r="R40" s="60" t="inlineStr">
+        <is>
+          <t>25/08/2026</t>
+        </is>
+      </c>
+      <c r="S40" s="60" t="inlineStr">
+        <is>
+          <t>16:14:00</t>
+        </is>
+      </c>
+      <c r="T40" s="60" t="inlineStr">
+        <is>
+          <t>LUARI - 27D1B044</t>
+        </is>
+      </c>
+      <c r="U40" s="60" t="inlineStr">
+        <is>
+          <t>atualizacao</t>
+        </is>
+      </c>
+      <c r="V40" s="60" t="n"/>
+      <c r="W40" s="60" t="inlineStr">
+        <is>
+          <t>527878</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>